<commit_message>
Edited Forms and New Form 2
</commit_message>
<xml_diff>
--- a/public/exel/sns_elem.xlsx
+++ b/public/exel/sns_elem.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\sbfp_ao_system\public\exel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B65595-EAFC-4E2B-AD22-4D4EA1C0D6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FEC04F0-F720-46EA-B669-6B93A34C2D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{5C1FB759-1B09-4FD4-91F7-CD6FCA4D472E}"/>
   </bookViews>
@@ -141,6 +141,15 @@
     <t>SBFP DepEd Focal</t>
   </si>
   <si>
+    <t>Approved by :</t>
+  </si>
+  <si>
+    <t>School Head</t>
+  </si>
+  <si>
+    <t>(School Head Name)</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Baseline (June) </t>
     </r>
@@ -152,17 +161,8 @@
         <color rgb="FF0000FF"/>
         <rFont val="Tahoma"/>
       </rPr>
-      <t>SY  2025 -2026</t>
+      <t>SY  2026 -2027</t>
     </r>
-  </si>
-  <si>
-    <t>Approved by :</t>
-  </si>
-  <si>
-    <t>School Head</t>
-  </si>
-  <si>
-    <t>(School Head Name)</t>
   </si>
 </sst>
 </file>
@@ -1193,57 +1193,26 @@
     <xf numFmtId="3" fontId="11" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1264,19 +1233,50 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1786,7 +1786,7 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="75" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B5" s="73"/>
       <c r="C5" s="73"/>
@@ -1841,93 +1841,93 @@
       <c r="Y6" s="1"/>
     </row>
     <row r="7" spans="1:25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="59"/>
-      <c r="D7" s="64" t="s">
+      <c r="C7" s="80"/>
+      <c r="D7" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="65"/>
-      <c r="F7" s="68" t="s">
+      <c r="E7" s="86"/>
+      <c r="F7" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="69"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="69"/>
-      <c r="J7" s="69"/>
-      <c r="K7" s="69"/>
-      <c r="L7" s="69"/>
-      <c r="M7" s="69"/>
-      <c r="N7" s="69"/>
-      <c r="O7" s="70"/>
-      <c r="P7" s="71" t="s">
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
+      <c r="I7" s="89"/>
+      <c r="J7" s="89"/>
+      <c r="K7" s="89"/>
+      <c r="L7" s="89"/>
+      <c r="M7" s="89"/>
+      <c r="N7" s="89"/>
+      <c r="O7" s="90"/>
+      <c r="P7" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="Q7" s="69"/>
-      <c r="R7" s="69"/>
-      <c r="S7" s="69"/>
-      <c r="T7" s="69"/>
-      <c r="U7" s="69"/>
-      <c r="V7" s="69"/>
-      <c r="W7" s="70"/>
-      <c r="X7" s="76" t="s">
+      <c r="Q7" s="89"/>
+      <c r="R7" s="89"/>
+      <c r="S7" s="89"/>
+      <c r="T7" s="89"/>
+      <c r="U7" s="89"/>
+      <c r="V7" s="89"/>
+      <c r="W7" s="90"/>
+      <c r="X7" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="Y7" s="77"/>
+      <c r="Y7" s="61"/>
     </row>
     <row r="8" spans="1:25">
-      <c r="A8" s="56"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="79" t="s">
+      <c r="A8" s="77"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="80"/>
-      <c r="H8" s="81" t="s">
+      <c r="G8" s="65"/>
+      <c r="H8" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="80"/>
-      <c r="J8" s="82" t="s">
+      <c r="I8" s="65"/>
+      <c r="J8" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="80"/>
-      <c r="L8" s="82" t="s">
+      <c r="K8" s="65"/>
+      <c r="L8" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="80"/>
-      <c r="N8" s="82" t="s">
+      <c r="M8" s="65"/>
+      <c r="N8" s="67" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="83"/>
-      <c r="P8" s="84" t="s">
+      <c r="O8" s="68"/>
+      <c r="P8" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="80"/>
-      <c r="R8" s="85" t="s">
+      <c r="Q8" s="65"/>
+      <c r="R8" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="80"/>
-      <c r="T8" s="86" t="s">
+      <c r="S8" s="65"/>
+      <c r="T8" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="U8" s="80"/>
-      <c r="V8" s="86" t="s">
+      <c r="U8" s="65"/>
+      <c r="V8" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="W8" s="83"/>
-      <c r="X8" s="78"/>
-      <c r="Y8" s="67"/>
+      <c r="W8" s="68"/>
+      <c r="X8" s="62"/>
+      <c r="Y8" s="63"/>
     </row>
     <row r="9" spans="1:25" ht="15" thickBot="1">
-      <c r="A9" s="57"/>
-      <c r="B9" s="62"/>
-      <c r="C9" s="63"/>
+      <c r="A9" s="78"/>
+      <c r="B9" s="83"/>
+      <c r="C9" s="84"/>
       <c r="D9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1996,7 +1996,7 @@
       </c>
     </row>
     <row r="10" spans="1:25" ht="15" thickTop="1">
-      <c r="A10" s="94" t="s">
+      <c r="A10" s="59" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -2086,7 +2086,7 @@
       </c>
     </row>
     <row r="11" spans="1:25">
-      <c r="A11" s="88"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="10" t="s">
         <v>22</v>
       </c>
@@ -2174,7 +2174,7 @@
       </c>
     </row>
     <row r="12" spans="1:25">
-      <c r="A12" s="89"/>
+      <c r="A12" s="54"/>
       <c r="B12" s="12" t="s">
         <v>23</v>
       </c>
@@ -2272,7 +2272,7 @@
       </c>
     </row>
     <row r="13" spans="1:25">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="52" t="s">
         <v>24</v>
       </c>
       <c r="B13" s="10" t="s">
@@ -2362,7 +2362,7 @@
       </c>
     </row>
     <row r="14" spans="1:25">
-      <c r="A14" s="88"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="10" t="s">
         <v>22</v>
       </c>
@@ -2450,7 +2450,7 @@
       </c>
     </row>
     <row r="15" spans="1:25">
-      <c r="A15" s="89"/>
+      <c r="A15" s="54"/>
       <c r="B15" s="12" t="s">
         <v>23</v>
       </c>
@@ -2548,7 +2548,7 @@
       </c>
     </row>
     <row r="16" spans="1:25">
-      <c r="A16" s="87" t="s">
+      <c r="A16" s="52" t="s">
         <v>25</v>
       </c>
       <c r="B16" s="10" t="s">
@@ -2638,7 +2638,7 @@
       </c>
     </row>
     <row r="17" spans="1:25">
-      <c r="A17" s="88"/>
+      <c r="A17" s="53"/>
       <c r="B17" s="10" t="s">
         <v>22</v>
       </c>
@@ -2726,7 +2726,7 @@
       </c>
     </row>
     <row r="18" spans="1:25">
-      <c r="A18" s="89"/>
+      <c r="A18" s="54"/>
       <c r="B18" s="12" t="s">
         <v>23</v>
       </c>
@@ -2824,7 +2824,7 @@
       </c>
     </row>
     <row r="19" spans="1:25">
-      <c r="A19" s="87" t="s">
+      <c r="A19" s="52" t="s">
         <v>26</v>
       </c>
       <c r="B19" s="10" t="s">
@@ -2914,7 +2914,7 @@
       </c>
     </row>
     <row r="20" spans="1:25">
-      <c r="A20" s="88"/>
+      <c r="A20" s="53"/>
       <c r="B20" s="10" t="s">
         <v>22</v>
       </c>
@@ -3002,7 +3002,7 @@
       </c>
     </row>
     <row r="21" spans="1:25">
-      <c r="A21" s="89"/>
+      <c r="A21" s="54"/>
       <c r="B21" s="12" t="s">
         <v>23</v>
       </c>
@@ -3100,7 +3100,7 @@
       </c>
     </row>
     <row r="22" spans="1:25">
-      <c r="A22" s="87" t="s">
+      <c r="A22" s="52" t="s">
         <v>27</v>
       </c>
       <c r="B22" s="10" t="s">
@@ -3190,7 +3190,7 @@
       </c>
     </row>
     <row r="23" spans="1:25">
-      <c r="A23" s="88"/>
+      <c r="A23" s="53"/>
       <c r="B23" s="10" t="s">
         <v>22</v>
       </c>
@@ -3278,7 +3278,7 @@
       </c>
     </row>
     <row r="24" spans="1:25">
-      <c r="A24" s="89"/>
+      <c r="A24" s="54"/>
       <c r="B24" s="12" t="s">
         <v>23</v>
       </c>
@@ -3376,7 +3376,7 @@
       </c>
     </row>
     <row r="25" spans="1:25">
-      <c r="A25" s="87" t="s">
+      <c r="A25" s="52" t="s">
         <v>28</v>
       </c>
       <c r="B25" s="10" t="s">
@@ -3466,7 +3466,7 @@
       </c>
     </row>
     <row r="26" spans="1:25">
-      <c r="A26" s="88"/>
+      <c r="A26" s="53"/>
       <c r="B26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3554,7 +3554,7 @@
       </c>
     </row>
     <row r="27" spans="1:25">
-      <c r="A27" s="89"/>
+      <c r="A27" s="54"/>
       <c r="B27" s="12" t="s">
         <v>23</v>
       </c>
@@ -3652,7 +3652,7 @@
       </c>
     </row>
     <row r="28" spans="1:25">
-      <c r="A28" s="87" t="s">
+      <c r="A28" s="52" t="s">
         <v>29</v>
       </c>
       <c r="B28" s="10" t="s">
@@ -3742,7 +3742,7 @@
       </c>
     </row>
     <row r="29" spans="1:25">
-      <c r="A29" s="88"/>
+      <c r="A29" s="53"/>
       <c r="B29" s="10" t="s">
         <v>22</v>
       </c>
@@ -3830,7 +3830,7 @@
       </c>
     </row>
     <row r="30" spans="1:25">
-      <c r="A30" s="89"/>
+      <c r="A30" s="54"/>
       <c r="B30" s="12" t="s">
         <v>23</v>
       </c>
@@ -3928,7 +3928,7 @@
       </c>
     </row>
     <row r="31" spans="1:25">
-      <c r="A31" s="87" t="s">
+      <c r="A31" s="52" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="10" t="s">
@@ -4018,7 +4018,7 @@
       </c>
     </row>
     <row r="32" spans="1:25">
-      <c r="A32" s="88"/>
+      <c r="A32" s="53"/>
       <c r="B32" s="10" t="s">
         <v>22</v>
       </c>
@@ -4106,7 +4106,7 @@
       </c>
     </row>
     <row r="33" spans="1:25" ht="15" thickBot="1">
-      <c r="A33" s="90"/>
+      <c r="A33" s="55"/>
       <c r="B33" s="33" t="s">
         <v>23</v>
       </c>
@@ -4204,7 +4204,7 @@
       </c>
     </row>
     <row r="34" spans="1:25">
-      <c r="A34" s="91" t="s">
+      <c r="A34" s="56" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="36" t="s">
@@ -4304,7 +4304,7 @@
       </c>
     </row>
     <row r="35" spans="1:25">
-      <c r="A35" s="92"/>
+      <c r="A35" s="57"/>
       <c r="B35" s="37" t="s">
         <v>22</v>
       </c>
@@ -4402,7 +4402,7 @@
       </c>
     </row>
     <row r="36" spans="1:25" ht="15" thickBot="1">
-      <c r="A36" s="93"/>
+      <c r="A36" s="58"/>
       <c r="B36" s="38" t="s">
         <v>23</v>
       </c>
@@ -4555,12 +4555,12 @@
     </row>
     <row r="39" spans="1:25" s="21" customFormat="1" ht="12">
       <c r="A39" s="20"/>
-      <c r="B39" s="54" t="s">
+      <c r="B39" s="94" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="54"/>
+      <c r="C39" s="94"/>
+      <c r="D39" s="94"/>
+      <c r="E39" s="94"/>
       <c r="F39" s="20"/>
       <c r="G39" s="20"/>
       <c r="H39" s="20"/>
@@ -4571,12 +4571,12 @@
       <c r="M39" s="20"/>
       <c r="N39" s="20"/>
       <c r="O39" s="20"/>
-      <c r="P39" s="54" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q39" s="54"/>
-      <c r="R39" s="54"/>
-      <c r="S39" s="54"/>
+      <c r="P39" s="94" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q39" s="94"/>
+      <c r="R39" s="94"/>
+      <c r="S39" s="94"/>
       <c r="T39" s="20"/>
       <c r="U39" s="20"/>
       <c r="V39" s="20"/>
@@ -4586,12 +4586,12 @@
     </row>
     <row r="40" spans="1:25" s="21" customFormat="1" ht="12">
       <c r="A40" s="20"/>
-      <c r="B40" s="53" t="s">
+      <c r="B40" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="C40" s="53"/>
-      <c r="D40" s="53"/>
-      <c r="E40" s="53"/>
+      <c r="C40" s="93"/>
+      <c r="D40" s="93"/>
+      <c r="E40" s="93"/>
       <c r="F40" s="20"/>
       <c r="G40" s="20"/>
       <c r="H40" s="20"/>
@@ -4602,12 +4602,12 @@
       <c r="M40" s="20"/>
       <c r="N40" s="20"/>
       <c r="O40" s="20"/>
-      <c r="P40" s="53" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q40" s="53"/>
-      <c r="R40" s="53"/>
-      <c r="S40" s="53"/>
+      <c r="P40" s="93" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q40" s="93"/>
+      <c r="R40" s="93"/>
+      <c r="S40" s="93"/>
       <c r="T40" s="20"/>
       <c r="U40" s="20"/>
       <c r="V40" s="20"/>
@@ -4617,12 +4617,12 @@
     </row>
     <row r="41" spans="1:25" s="21" customFormat="1" ht="12">
       <c r="A41" s="20"/>
-      <c r="B41" s="52" t="s">
+      <c r="B41" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
+      <c r="C41" s="92"/>
+      <c r="D41" s="92"/>
+      <c r="E41" s="92"/>
       <c r="F41" s="20"/>
       <c r="G41" s="20"/>
       <c r="H41" s="20"/>
@@ -4633,12 +4633,12 @@
       <c r="M41" s="20"/>
       <c r="N41" s="20"/>
       <c r="O41" s="20"/>
-      <c r="P41" s="52" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q41" s="52"/>
-      <c r="R41" s="52"/>
-      <c r="S41" s="52"/>
+      <c r="P41" s="92" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q41" s="92"/>
+      <c r="R41" s="92"/>
+      <c r="S41" s="92"/>
       <c r="T41" s="20"/>
       <c r="U41" s="20"/>
       <c r="V41" s="20"/>
@@ -30541,15 +30541,22 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="P41:S41"/>
+    <mergeCell ref="P40:S40"/>
+    <mergeCell ref="P39:S39"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:C9"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="F7:O7"/>
+    <mergeCell ref="P7:W7"/>
+    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A2:Y2"/>
+    <mergeCell ref="A3:Y3"/>
+    <mergeCell ref="A4:Y4"/>
+    <mergeCell ref="A5:Y5"/>
     <mergeCell ref="X7:Y8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="H8:I8"/>
@@ -30560,22 +30567,15 @@
     <mergeCell ref="R8:S8"/>
     <mergeCell ref="T8:U8"/>
     <mergeCell ref="V8:W8"/>
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A3:Y3"/>
-    <mergeCell ref="A4:Y4"/>
-    <mergeCell ref="A5:Y5"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:C9"/>
-    <mergeCell ref="D7:E8"/>
-    <mergeCell ref="F7:O7"/>
-    <mergeCell ref="P7:W7"/>
-    <mergeCell ref="P41:S41"/>
-    <mergeCell ref="P40:S40"/>
-    <mergeCell ref="P39:S39"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="78" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>